<commit_message>
daily work report | 31-03-2026
</commit_message>
<xml_diff>
--- a/MPR/Role wise/Technical Support/Feb'26/Individual_MPR (Haripriya).xlsx
+++ b/MPR/Role wise/Technical Support/Feb'26/Individual_MPR (Haripriya).xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="76">
   <si>
     <t>SR#</t>
   </si>
@@ -74,27 +74,15 @@
     <t>5th feb</t>
   </si>
   <si>
-    <t>4th feb</t>
-  </si>
-  <si>
     <t xml:space="preserve">TMS </t>
   </si>
   <si>
     <t>10th feb</t>
   </si>
   <si>
-    <t xml:space="preserve">7th feb </t>
-  </si>
-  <si>
     <t xml:space="preserve">worked on contact person creation &amp; updation  and validations in the field </t>
   </si>
   <si>
-    <t xml:space="preserve">8th feb </t>
-  </si>
-  <si>
-    <t xml:space="preserve">9th feb </t>
-  </si>
-  <si>
     <t xml:space="preserve">On leave due to personal reasons </t>
   </si>
   <si>
@@ -117,9 +105,6 @@
   </si>
   <si>
     <t>Worked on CRP-EP App- Worked on the CRP EP app to analyze fields whose data is not being recorded in the backend database, and identified new fields that need to be added to the backend.</t>
-  </si>
-  <si>
-    <t>12th feb</t>
   </si>
   <si>
     <t>Implemented language conversion in the Existing Form module, covering the Investment Details section and the Loan &amp; Subsidy Details section, including all related loan and subsidy components.</t>
@@ -176,16 +161,7 @@
     <t xml:space="preserve">week off </t>
   </si>
   <si>
-    <t>16th feb</t>
-  </si>
-  <si>
     <t>Harpriya</t>
-  </si>
-  <si>
-    <t>17th feb</t>
-  </si>
-  <si>
-    <t>18th feb</t>
   </si>
   <si>
     <t>Worked on crp-ep app- Worked on the complete Loan Details and Subsidy Details sections, restructuring the API data storage flow as per the updated backend requirements.
@@ -199,9 +175,6 @@
 Also implemented the Subsidy section with fields like Subsidy Taken (Yes/No), institution name, and description, making sure all details are properly validated, mapped, and stored in the backend as per the updated API format.</t>
   </si>
   <si>
-    <t>19th feb</t>
-  </si>
-  <si>
     <t>Worked on CRP-EP App-Worked on the Enterprise Shop section, aligning frontend fields with the updated API structure and ensuring data is correctly sent and mapped to the appropriate backend fields.
 Implemented and integrated the Enterprise Media fields, ensuring proper file handling and accurate API data submission as per the revised backend format.
 Modified the entire Enterprise Product section according to the updated API, including proper mapping and submission of all product-related fields along with media attachments.
@@ -212,12 +185,6 @@
 Additionally, modified the entire Enterprise Product section to align with the updated APIs, including proper mapping of all product-related fields and media attachments. Worked on the Cadre and Cadre Designation fields as well, ensuring correct data transmission and successful API submission based on the new structure.</t>
   </si>
   <si>
-    <t>20th feb</t>
-  </si>
-  <si>
-    <t>21st feb</t>
-  </si>
-  <si>
     <t xml:space="preserve">weekoff Sunday </t>
   </si>
   <si>
@@ -234,30 +201,15 @@
     <t>Compensatory leave due to office work on Sunday (08-02-26)</t>
   </si>
   <si>
-    <t xml:space="preserve">Worked on TMS home page UI along with responsoveness </t>
-  </si>
-  <si>
     <t>competed</t>
   </si>
   <si>
-    <t>24th feb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25th feb </t>
-  </si>
-  <si>
     <t xml:space="preserve">worked on the header section and its pages and subpages </t>
   </si>
   <si>
-    <t xml:space="preserve">26th feb </t>
-  </si>
-  <si>
     <t xml:space="preserve">worked on the header section and its pages and subpages LDMS, enterprise tracking, monitoring &amp; analysis </t>
   </si>
   <si>
-    <t xml:space="preserve">27th feb </t>
-  </si>
-  <si>
     <t xml:space="preserve"> header section suboptions- Dashboard - suboptions ,Resource centre suboptions, login button UI along with responsiveness </t>
   </si>
   <si>
@@ -265,18 +217,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dashboard  UI part added graph chart for the analytics  and worked on the card UI along with daashboard structure </t>
-  </si>
-  <si>
-    <t>Worked on the TMS, including the header section, the About Us page and its subpages, the Our Services section and its subpages, Beneficiary Profiling, and User Management, while also improving their responsiveness.</t>
-  </si>
-  <si>
-    <t>Worked on TMS, focusing on the header section options including LDMS, Enterprise Tracking, and Monitoring &amp; Analysis.</t>
-  </si>
-  <si>
-    <t>Worked on TMS, including the header section sub-options such as Dashboard (with its sub-options), Resource Centre sub-options, and the Login button UI, along with improving responsiveness</t>
-  </si>
-  <si>
-    <t>Worked on the TMS Dashboard UI by adding graph charts for analytics, designing card components, and improving the overall dashboard structure</t>
   </si>
   <si>
     <t xml:space="preserve">Worked on the UI part of the TMS home page including all the homepage sections </t>
@@ -325,6 +265,36 @@
 Developed and integrated new fields including dependent dropdowns, multi-selects, and conditional inputs with proper state management.
 Implemented smooth frontend interactions with live validation and consistent data binding for better user experience.
 Conducted thorough testing, debugging, and performance optimization to ensure stable and efficient form functionality.</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10th feb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ongoing </t>
+  </si>
+  <si>
+    <t>ongoing</t>
+  </si>
+  <si>
+    <t>28th feb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked on Pragati Setu home page UI along with responsoveness </t>
+  </si>
+  <si>
+    <t>Worked on the Pragati Setu, including the header section, the About Us page and its subpages, the Our Services section and its subpages, Beneficiary Profiling, and User Management, while also improving their responsiveness.</t>
+  </si>
+  <si>
+    <t>Worked on Pragati Setu, focusing on the header section options including LDMS, Enterprise Tracking, and Monitoring &amp; Analysis.</t>
+  </si>
+  <si>
+    <t>Worked on Pragati Setu, including the header section sub-options such as Dashboard (with its sub-options), Resource Centre sub-options, and the Login button UI, along with improving responsiveness</t>
+  </si>
+  <si>
+    <t>Worked on the Pragati Setu Dashboard UI by adding graph charts for analytics, designing card components, and improving the overall dashboard structure</t>
   </si>
 </sst>
 </file>
@@ -464,6 +434,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -482,7 +453,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -801,21 +771,21 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>11</v>
@@ -838,7 +808,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>11</v>
@@ -861,22 +831,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -884,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>11</v>
@@ -899,43 +869,43 @@
         <v>10</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="B7" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -943,22 +913,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>11</v>
+        <v>32</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -966,22 +936,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>11</v>
+        <v>32</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
@@ -989,22 +959,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>18</v>
-      </c>
       <c r="F11" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1012,22 +982,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="114" customHeight="1" x14ac:dyDescent="0.3">
@@ -1035,22 +1005,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
@@ -1058,71 +1028,71 @@
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="B15" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="7">
         <v>15</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="B16" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
     </row>
     <row r="17" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E17" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1130,22 +1100,22 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
@@ -1153,22 +1123,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E19" t="s">
         <v>48</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
@@ -1176,22 +1146,22 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1199,22 +1169,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1222,173 +1192,173 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="7">
         <v>22</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
+      <c r="B23" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A24" s="7">
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
         <v>11</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="15">
+      <c r="A25" s="9">
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="15">
+      <c r="A26" s="9">
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="15">
+      <c r="A27" s="9">
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>73</v>
       </c>
       <c r="C27" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="15">
+      <c r="A28" s="9">
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="15">
+      <c r="A29" s="9">
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>